<commit_message>
Update numerical data for week of 06.15.2026
</commit_message>
<xml_diff>
--- a/jdca_weekly_metrics_asof_2026-06-15.xlsx
+++ b/jdca_weekly_metrics_asof_2026-06-15.xlsx
@@ -570,7 +570,7 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1007640969216</v>
+        <v>1006936588288</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -601,7 +601,7 @@
         <v>28.12</v>
       </c>
       <c r="T2" t="n">
-        <v>40.183853</v>
+        <v>40.15576</v>
       </c>
       <c r="U2" t="n">
         <v>1.497</v>
@@ -642,7 +642,7 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>193926201344</v>
+        <v>194125512704</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -673,7 +673,7 @@
         <v>4.24</v>
       </c>
       <c r="T3" t="n">
-        <v>10.326652</v>
+        <v>10.337265</v>
       </c>
       <c r="U3" t="n">
         <v>0.788</v>
@@ -714,7 +714,7 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>105313861632</v>
+        <v>105493397504</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -745,7 +745,7 @@
         <v>2.29</v>
       </c>
       <c r="T4" t="n">
-        <v>19.21179</v>
+        <v>19.244541</v>
       </c>
       <c r="U4" t="n">
         <v>1.005</v>
@@ -786,7 +786,7 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>114321571840</v>
+        <v>114584264704</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -817,7 +817,7 @@
         <v>16.85</v>
       </c>
       <c r="T5" t="n">
-        <v>26.73175</v>
+        <v>26.793175</v>
       </c>
       <c r="U5" t="n">
         <v>3.023</v>
@@ -938,7 +938,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>5061099520</v>
+        <v>5072917504</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1234,7 +1234,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>280423648</v>
+        <v>280531520</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1312,7 +1312,7 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>5000292</v>
+        <v>4999200</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1390,7 +1390,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>403994784</v>
+        <v>401289440</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1852,7 +1852,7 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>1415080320</v>
+        <v>1419658240</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1930,7 +1930,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>8315284</v>
+        <v>8317503</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -2008,7 +2008,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>264754240</v>
+        <v>265518384</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Fill in missing values for several companies for week of 06.15.2026
</commit_message>
<xml_diff>
--- a/jdca_weekly_metrics_asof_2026-06-15.xlsx
+++ b/jdca_weekly_metrics_asof_2026-06-15.xlsx
@@ -570,24 +570,31 @@
         <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>1006936588288</v>
+        <v>1007085486080</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
           <t>Large-cap</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="n">
+        <v>1129.35</v>
+      </c>
       <c r="J2" t="n">
         <v>619.3983893784804</v>
       </c>
       <c r="K2" t="n">
         <v>1182.72998046875</v>
       </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>-0.003221535745807635</v>
+      </c>
+      <c r="N2" t="n">
+        <v>-3.482153574580764</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.05443640086150614</v>
+      </c>
       <c r="P2" t="n">
         <v>3198890.33</v>
       </c>
@@ -601,7 +608,7 @@
         <v>28.12</v>
       </c>
       <c r="T2" t="n">
-        <v>40.15576</v>
+        <v>40.1617</v>
       </c>
       <c r="U2" t="n">
         <v>1.497</v>
@@ -642,24 +649,31 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
-        <v>194125512704</v>
+        <v>193859764224</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
           <t>Large-cap</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="n">
+        <v>43.92</v>
+      </c>
       <c r="J3" t="n">
         <v>34.58171819384536</v>
       </c>
       <c r="K3" t="n">
         <v>77.68348832838186</v>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
+      <c r="L3" t="n">
+        <v>0.0009115770282588365</v>
+      </c>
+      <c r="N3" t="n">
+        <v>-3.068842297174116</v>
+      </c>
+      <c r="O3" t="n">
+        <v>-0.1051348181374939</v>
+      </c>
       <c r="P3" t="n">
         <v>19582796.93</v>
       </c>
@@ -673,7 +687,7 @@
         <v>4.24</v>
       </c>
       <c r="T3" t="n">
-        <v>10.337265</v>
+        <v>10.323113</v>
       </c>
       <c r="U3" t="n">
         <v>0.788</v>
@@ -714,24 +728,31 @@
         <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>105493397504</v>
+        <v>105373712384</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
           <t>Large-cap</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="n">
+        <v>43.8</v>
+      </c>
       <c r="J4" t="n">
         <v>41.0430664238207</v>
       </c>
       <c r="K4" t="n">
         <v>49.91109967191108</v>
       </c>
-      <c r="L4" t="inlineStr"/>
-      <c r="M4" t="inlineStr"/>
-      <c r="N4" t="inlineStr"/>
-      <c r="O4" t="inlineStr"/>
+      <c r="L4" t="n">
+        <v>-0.01016949152542379</v>
+      </c>
+      <c r="N4" t="n">
+        <v>-4.176949152542379</v>
+      </c>
+      <c r="O4" t="n">
+        <v>-0.04601943026435751</v>
+      </c>
       <c r="P4" t="n">
         <v>3462239.72</v>
       </c>
@@ -745,7 +766,7 @@
         <v>2.29</v>
       </c>
       <c r="T4" t="n">
-        <v>19.244541</v>
+        <v>19.222708</v>
       </c>
       <c r="U4" t="n">
         <v>1.005</v>
@@ -786,24 +807,31 @@
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>114584264704</v>
+        <v>114449752064</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
           <t>Large-cap</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="n">
+        <v>450.46</v>
+      </c>
       <c r="J5" t="n">
         <v>362.5</v>
       </c>
       <c r="K5" t="n">
         <v>507.9200134277344</v>
       </c>
-      <c r="L5" t="inlineStr"/>
-      <c r="M5" t="inlineStr"/>
-      <c r="N5" t="inlineStr"/>
-      <c r="O5" t="inlineStr"/>
+      <c r="L5" t="n">
+        <v>0.01242892140336682</v>
+      </c>
+      <c r="N5" t="n">
+        <v>-1.917107859663318</v>
+      </c>
+      <c r="O5" t="n">
+        <v>-0.006396858407079598</v>
+      </c>
       <c r="P5" t="n">
         <v>1330408.32</v>
       </c>
@@ -817,7 +845,7 @@
         <v>16.85</v>
       </c>
       <c r="T5" t="n">
-        <v>26.793175</v>
+        <v>26.76172</v>
       </c>
       <c r="U5" t="n">
         <v>3.023</v>
@@ -877,7 +905,6 @@
       <c r="L6" t="n">
         <v>-0.03834536809699007</v>
       </c>
-      <c r="M6" t="inlineStr"/>
       <c r="N6" t="n">
         <v>-6.994259790635371</v>
       </c>
@@ -938,7 +965,7 @@
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>5072917504</v>
+        <v>5084242944</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -957,7 +984,6 @@
       <c r="L7" t="n">
         <v>0.01957368538948723</v>
       </c>
-      <c r="M7" t="inlineStr"/>
       <c r="N7" t="n">
         <v>-1.202354441987641</v>
       </c>
@@ -976,7 +1002,6 @@
       <c r="S7" t="n">
         <v>-6.17</v>
       </c>
-      <c r="T7" t="inlineStr"/>
       <c r="U7" t="n">
         <v>17.965</v>
       </c>
@@ -1016,7 +1041,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>786173760</v>
+        <v>787565184</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1035,7 +1060,6 @@
       <c r="L8" t="n">
         <v>0.05947949591400192</v>
       </c>
-      <c r="M8" t="inlineStr"/>
       <c r="N8" t="n">
         <v>2.788226610463829</v>
       </c>
@@ -1054,7 +1078,6 @@
       <c r="S8" t="n">
         <v>-0.92</v>
       </c>
-      <c r="T8" t="inlineStr"/>
       <c r="U8" t="n">
         <v>1.295</v>
       </c>
@@ -1094,24 +1117,31 @@
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>960250944</v>
+        <v>961565120</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
           <t>Small-cap</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>2.83</v>
+      </c>
       <c r="J9" t="n">
         <v>2.309999942779541</v>
       </c>
       <c r="K9" t="n">
         <v>4.420000076293945</v>
       </c>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
+      <c r="L9" t="n">
+        <v>0.04044117647058809</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.8841176470588088</v>
+      </c>
+      <c r="O9" t="n">
+        <v>-0.0811684911032029</v>
+      </c>
       <c r="P9" t="n">
         <v>115242.08</v>
       </c>
@@ -1124,7 +1154,6 @@
       <c r="S9" t="n">
         <v>-0.63</v>
       </c>
-      <c r="T9" t="inlineStr"/>
       <c r="U9" t="n">
         <v>1.68</v>
       </c>
@@ -1171,17 +1200,24 @@
           <t>Small-cap</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>1.25</v>
+      </c>
       <c r="J10" t="n">
         <v>0.6899999976158142</v>
       </c>
       <c r="K10" t="n">
         <v>2.089999914169312</v>
       </c>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
+      <c r="L10" t="n">
+        <v>-0.01574803149606296</v>
+      </c>
+      <c r="N10" t="n">
+        <v>-4.734803149606297</v>
+      </c>
+      <c r="O10" t="n">
+        <v>-0.2514969008264463</v>
+      </c>
       <c r="P10" t="n">
         <v>1183970.71</v>
       </c>
@@ -1194,7 +1230,6 @@
       <c r="S10" t="n">
         <v>-0.29</v>
       </c>
-      <c r="T10" t="inlineStr"/>
       <c r="U10" t="n">
         <v>6.893</v>
       </c>
@@ -1234,7 +1269,7 @@
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>280531520</v>
+        <v>280450624</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1253,7 +1288,6 @@
       <c r="L11" t="n">
         <v>-0.2246376404715194</v>
       </c>
-      <c r="M11" t="inlineStr"/>
       <c r="N11" t="n">
         <v>-25.6234870280883</v>
       </c>
@@ -1272,7 +1306,6 @@
       <c r="S11" t="n">
         <v>-0.63</v>
       </c>
-      <c r="T11" t="inlineStr"/>
       <c r="U11" t="n">
         <v>3.929</v>
       </c>
@@ -1312,7 +1345,7 @@
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>4999200</v>
+        <v>4995921</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1331,7 +1364,6 @@
       <c r="L12" t="n">
         <v>-0.2742176068744142</v>
       </c>
-      <c r="M12" t="inlineStr"/>
       <c r="N12" t="n">
         <v>-30.58148366837779</v>
       </c>
@@ -1350,7 +1382,6 @@
       <c r="S12" t="n">
         <v>-5.06</v>
       </c>
-      <c r="T12" t="inlineStr"/>
       <c r="U12" t="n">
         <v>5.607</v>
       </c>
@@ -1390,7 +1421,7 @@
         <v>1</v>
       </c>
       <c r="G13" t="n">
-        <v>401289440</v>
+        <v>403092992</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1409,7 +1440,6 @@
       <c r="L13" t="n">
         <v>0.08490569644994705</v>
       </c>
-      <c r="M13" t="inlineStr"/>
       <c r="N13" t="n">
         <v>5.330846664058342</v>
       </c>
@@ -1428,7 +1458,6 @@
       <c r="S13" t="n">
         <v>-1.14</v>
       </c>
-      <c r="T13" t="inlineStr"/>
       <c r="U13" t="n">
         <v>10.249</v>
       </c>
@@ -1468,11 +1497,11 @@
         <v>1</v>
       </c>
       <c r="G14" t="n">
-        <v>298209984</v>
+        <v>303562464</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Micro-cap</t>
+          <t>Small-cap</t>
         </is>
       </c>
       <c r="I14" t="n">
@@ -1487,7 +1516,6 @@
       <c r="L14" t="n">
         <v>0.147058819404523</v>
       </c>
-      <c r="M14" t="inlineStr"/>
       <c r="N14" t="n">
         <v>11.54615895951594</v>
       </c>
@@ -1506,7 +1534,6 @@
       <c r="S14" t="n">
         <v>-0.58</v>
       </c>
-      <c r="T14" t="inlineStr"/>
       <c r="U14" t="n">
         <v>11.447</v>
       </c>
@@ -1553,17 +1580,24 @@
           <t>Micro-cap</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>0.11</v>
+      </c>
       <c r="J15" t="n">
         <v>0.09000000357627869</v>
       </c>
       <c r="K15" t="n">
         <v>0.1599999964237213</v>
       </c>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>-3.16</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0.2222219999999999</v>
+      </c>
       <c r="P15" t="n">
         <v>40047.25274725275</v>
       </c>
@@ -1576,7 +1610,6 @@
       <c r="S15" t="n">
         <v>-0.03</v>
       </c>
-      <c r="T15" t="inlineStr"/>
       <c r="U15" t="n">
         <v>0.139</v>
       </c>
@@ -1635,7 +1668,6 @@
       <c r="L16" t="n">
         <v>-0.01234566720224994</v>
       </c>
-      <c r="M16" t="inlineStr"/>
       <c r="N16" t="n">
         <v>-4.394289701161358</v>
       </c>
@@ -1654,7 +1686,6 @@
       <c r="S16" t="n">
         <v>-2.16</v>
       </c>
-      <c r="T16" t="inlineStr"/>
       <c r="U16" t="n">
         <v>0.759</v>
       </c>
@@ -1713,7 +1744,6 @@
       <c r="L17" t="n">
         <v>-0.2014562884311067</v>
       </c>
-      <c r="M17" t="inlineStr"/>
       <c r="N17" t="n">
         <v>-23.30535182404704</v>
       </c>
@@ -1793,7 +1823,6 @@
       <c r="L18" t="n">
         <v>-0.02597402453787323</v>
       </c>
-      <c r="M18" t="inlineStr"/>
       <c r="N18" t="n">
         <v>-5.757125434723687</v>
       </c>
@@ -1812,7 +1841,6 @@
       <c r="S18" t="n">
         <v>-0.43</v>
       </c>
-      <c r="T18" t="inlineStr"/>
       <c r="U18" t="n">
         <v>5.157</v>
       </c>
@@ -1852,7 +1880,7 @@
         <v>1</v>
       </c>
       <c r="G19" t="n">
-        <v>1419658240</v>
+        <v>1421438464</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1871,7 +1899,6 @@
       <c r="L19" t="n">
         <v>0.03022663611248455</v>
       </c>
-      <c r="M19" t="inlineStr"/>
       <c r="N19" t="n">
         <v>-0.1370593696879085</v>
       </c>
@@ -1890,7 +1917,6 @@
       <c r="S19" t="n">
         <v>-0.5600000000000001</v>
       </c>
-      <c r="T19" t="inlineStr"/>
       <c r="U19" t="n">
         <v>4.181</v>
       </c>
@@ -1930,7 +1956,7 @@
         <v>1</v>
       </c>
       <c r="G20" t="n">
-        <v>8317503</v>
+        <v>8243569</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1949,7 +1975,6 @@
       <c r="L20" t="n">
         <v>0.1016871625979778</v>
       </c>
-      <c r="M20" t="inlineStr"/>
       <c r="N20" t="n">
         <v>7.00899327886142</v>
       </c>
@@ -1968,7 +1993,6 @@
       <c r="S20" t="n">
         <v>-2.07</v>
       </c>
-      <c r="T20" t="inlineStr"/>
       <c r="U20" t="n">
         <v>19.694</v>
       </c>
@@ -2008,7 +2032,7 @@
         <v>1</v>
       </c>
       <c r="G21" t="n">
-        <v>265518384</v>
+        <v>266683920</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -2027,7 +2051,6 @@
       <c r="L21" t="n">
         <v>-0.04189940227528577</v>
       </c>
-      <c r="M21" t="inlineStr"/>
       <c r="N21" t="n">
         <v>-7.349663208464941</v>
       </c>
@@ -2046,7 +2069,6 @@
       <c r="S21" t="n">
         <v>-0.77</v>
       </c>
-      <c r="T21" t="inlineStr"/>
       <c r="U21" t="n">
         <v>8.439</v>
       </c>
@@ -2105,7 +2127,6 @@
       <c r="L22" t="n">
         <v>0.05062079344651793</v>
       </c>
-      <c r="M22" t="inlineStr"/>
       <c r="N22" t="n">
         <v>1.902356363715429</v>
       </c>
@@ -2124,8 +2145,6 @@
       <c r="S22" t="n">
         <v>-0.9</v>
       </c>
-      <c r="T22" t="inlineStr"/>
-      <c r="U22" t="inlineStr"/>
       <c r="V22" t="inlineStr">
         <is>
           <t>[[1745532000000, 4.502], [1746136800000, 4.9603], [1746741600000, 5.1054], [1747346400000, 4.9951], [1747951200000, 4.1423], [1748556000000, 4.2757], [1749160800000, 4.0263], [1749765600000, 4.2003], [1750370400000, 4.3686], [1750975200000, 4.3628], [1751580000000, 4.386], [1752184800000, 4.3628], [1752789600000, 4.7863], [1753394400000, 8.8183], [1753999200000, 7.7741], [1754604000000, 7.7741], [1755208800000, 11.4174], [1755813600000, 10.3267], [1756418400000, 9.6074], [1757023200000, 9.3173], [1757628000000, 9.5029], [1758232800000, 8.8183], [1758837600000, 8.4702], [1759442400000, 8.9228], [1760047200000, 11.313], [1760652000000, 11.4522], [1761256800000, 10.3499], [1761865200000, 10.1179], [1762470000000, 10.0715], [1763074800000, 10.3035], [1763679600000, 9.0272], [1764284400000, 9.3869], [1764889200000, 8.7487], [1765494000000, 8.1222], [1766098800000, 7.6232], [1766703600000, 7.3796], [1767308400000, 7.8089], [1767913200000, 6.9618], [1768518000000, 7.0199], [1769122800000, 7.5652], [1769727600000, 7.426], [1770332400000, 7.5768], [1770937200000, 7.4028], [1771542000000, 8.1222], [1772146800000, 7.7741], [1772751600000, 7.3099], [1773356400000, 6.8806], [1773961200000, 6.2657], [1774566000000, 5.2968], [1775167200000, 5.3838], [1775772000000, 5.472], [1776376800000, 5.9872], [1776981600000, 5.3815], [1777586400000, 5.6623], [1778191200000, 5.5532], [1778796000000, 5.6878], [1779400800000, 5.5811], [1780005600000, 5.725], [1780610400000, 4.9661], [1781215200000, 4.9661], [1781820000000, 5.1054]]</t>

</xml_diff>